<commit_message>
Refresh monster art and number monster entries sequentially
</commit_message>
<xml_diff>
--- a/Excel/moster.xlsx
+++ b/Excel/moster.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>tc={F70A43C4-509D-4B69-97A6-6DA2FFDBFBEC}</author>
+    <author>tc={5E0FA19B-CBDA-4150-A5F3-6D94AFC8F731}</author>
   </authors>
   <commentList>
     <comment ref="J1" authorId="0">
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
   <si>
     <t/>
   </si>
@@ -381,6 +381,81 @@
   </si>
   <si>
     <t>monster_02_d_2</t>
+  </si>
+  <si>
+    <t>灰鼠</t>
+  </si>
+  <si>
+    <t>灰黑色的鼠怪，背部生有短刺。</t>
+  </si>
+  <si>
+    <t>monster_03_a_1</t>
+  </si>
+  <si>
+    <t>monster_03_a_2</t>
+  </si>
+  <si>
+    <t>沙鼠</t>
+  </si>
+  <si>
+    <t>浅黄色的鼠怪，背部轮廓呈短刺状。</t>
+  </si>
+  <si>
+    <t>monster_03_b_1</t>
+  </si>
+  <si>
+    <t>monster_03_b_2</t>
+  </si>
+  <si>
+    <t>赤焰鼠</t>
+  </si>
+  <si>
+    <t>深红色的鼠怪，身侧带有橙黄色火焰状纹理。</t>
+  </si>
+  <si>
+    <t>monster_03_c_1</t>
+  </si>
+  <si>
+    <t>monster_03_c_2</t>
+  </si>
+  <si>
+    <t>晶背鼠</t>
+  </si>
+  <si>
+    <t>淡紫色的鼠怪，背部带有青蓝色晶体。</t>
+  </si>
+  <si>
+    <t>monster_03_d_1</t>
+  </si>
+  <si>
+    <t>monster_03_d_2</t>
+  </si>
+  <si>
+    <t>赤冠史莱姆</t>
+  </si>
+  <si>
+    <t>暗红色的大体型史莱姆，头顶生有赤红冠状突起。</t>
+  </si>
+  <si>
+    <t>monster_04_a_1</t>
+  </si>
+  <si>
+    <t>双生史莱姆</t>
+  </si>
+  <si>
+    <t>绿色的大体型史莱姆，身体上并列两张面孔。</t>
+  </si>
+  <si>
+    <t>monster_04_b_1</t>
+  </si>
+  <si>
+    <t>巨牙鼠</t>
+  </si>
+  <si>
+    <t>青蓝色的大体型鼠怪，口部生有长牙。</t>
+  </si>
+  <si>
+    <t>monster_04_c_1</t>
   </si>
 </sst>
 </file>
@@ -570,7 +645,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <tc2018:personList xmlns:tc2018="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="tc2018">
-  <tc2018:person displayName="空羽灵" id="{76EB59D8-A0D6-44AF-B4E5-0DEE303F7386}"/>
+  <tc2018:person displayName="空羽灵" id="{6C229CA3-6AF3-42F9-A7BA-A6CA3512C066}"/>
 </tc2018:personList>
 </file>
 
@@ -769,7 +844,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="">
-  <threadedComment ref="J1" dT="2026-10-08T14:11:22Z" personId="{76EB59D8-A0D6-44AF-B4E5-0DEE303F7386}" id="{F70A43C4-509D-4B69-97A6-6DA2FFDBFBEC}">
+  <threadedComment ref="J1" dT="2026-10-08T14:11:22Z" personId="{6C229CA3-6AF3-42F9-A7BA-A6CA3512C066}" id="{5E0FA19B-CBDA-4150-A5F3-6D94AFC8F731}">
     <text>1=城镇
 2=黑松林
 3=石牙矿洞
@@ -968,7 +1043,7 @@
         <v>1000</v>
       </c>
       <c r="L4" s="24" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="M4" s="24">
         <v>3</v>
@@ -985,34 +1060,34 @@
         <v>2</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D5" s="25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" s="25">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="F5" s="25">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="G5" s="25">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="H5" s="17">
         <v>0</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="K5" s="25">
-        <v>800</v>
+        <v>1000</v>
       </c>
       <c r="L5" s="24" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="M5" s="24">
         <v>3</v>
@@ -1026,37 +1101,37 @@
     <row r="6" spans="1:28" ht="39.95" customHeight="1">
       <c r="A6" s="17" t="s"/>
       <c r="B6" s="25">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="D6" s="25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" s="25">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="F6" s="25">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="G6" s="25">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H6" s="17">
         <v>0</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="K6" s="25">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="L6" s="24" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="M6" s="24">
         <v>3</v>
@@ -1070,37 +1145,37 @@
     <row r="7" spans="1:28" ht="39.95" customHeight="1">
       <c r="A7" s="17" t="s"/>
       <c r="B7" s="25">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="D7" s="25">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E7" s="25">
-        <v>30</v>
+        <v>72</v>
       </c>
       <c r="F7" s="25">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="G7" s="25">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H7" s="17">
         <v>0</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="K7" s="25">
-        <v>700</v>
+        <v>600</v>
       </c>
       <c r="L7" s="24" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="M7" s="24">
         <v>3</v>
@@ -1114,37 +1189,37 @@
     <row r="8" spans="1:28" ht="39.95" customHeight="1">
       <c r="A8" s="17" t="s"/>
       <c r="B8" s="25">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="D8" s="25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8" s="25">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="F8" s="25">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="G8" s="25">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H8" s="17">
         <v>0</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="K8" s="25">
         <v>800</v>
       </c>
       <c r="L8" s="24" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="M8" s="24">
         <v>3</v>
@@ -1158,37 +1233,37 @@
     <row r="9" spans="1:28" ht="39.95" customHeight="1">
       <c r="A9" s="17" t="s"/>
       <c r="B9" s="25">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="D9" s="25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" s="25">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F9" s="25">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="G9" s="25">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="H9" s="17">
         <v>0</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="J9" s="10" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="K9" s="25">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="L9" s="24" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="M9" s="24">
         <v>3</v>
@@ -1200,37 +1275,37 @@
     <row r="10" spans="1:13" ht="39.95" customHeight="1">
       <c r="A10" s="17" t="s"/>
       <c r="B10" s="25">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D10" s="25">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" s="25">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="F10" s="25">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="G10" s="25">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="H10" s="17">
         <v>0</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="K10" s="25">
         <v>600</v>
       </c>
       <c r="L10" s="24" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="M10" s="24">
         <v>3</v>
@@ -1239,7 +1314,7 @@
     <row r="11" spans="1:13" ht="39.95" customHeight="1">
       <c r="A11" s="17" t="s"/>
       <c r="B11" s="25">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>111</v>
@@ -1263,7 +1338,7 @@
         <v>112</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="K11" s="25">
         <v>800</v>
@@ -1277,108 +1352,276 @@
     </row>
     <row r="12" spans="1:13" ht="39.95" customHeight="1">
       <c r="A12" s="17" t="s"/>
-      <c r="B12" s="25" t="s"/>
-      <c r="C12" s="10" t="s"/>
-      <c r="D12" s="25" t="s"/>
-      <c r="E12" s="25" t="s"/>
-      <c r="F12" s="25" t="s"/>
-      <c r="G12" s="25" t="s"/>
-      <c r="H12" s="17" t="s"/>
-      <c r="I12" s="10" t="s"/>
-      <c r="J12" s="10" t="s"/>
-      <c r="K12" s="25" t="s"/>
-      <c r="L12" s="24" t="s"/>
-      <c r="M12" s="24" t="s"/>
+      <c r="B12" s="25">
+        <v>9</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="D12" s="25">
+        <v>1</v>
+      </c>
+      <c r="E12" s="25">
+        <v>18</v>
+      </c>
+      <c r="F12" s="25">
+        <v>5</v>
+      </c>
+      <c r="G12" s="25">
+        <v>1</v>
+      </c>
+      <c r="H12" s="17">
+        <v>0</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="J12" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="K12" s="25">
+        <v>1000</v>
+      </c>
+      <c r="L12" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="M12" s="24">
+        <v>3</v>
+      </c>
     </row>
     <row r="13" spans="1:13" ht="39.95" customHeight="1">
       <c r="A13" s="17" t="s"/>
-      <c r="B13" s="25" t="s"/>
-      <c r="C13" s="10" t="s"/>
-      <c r="D13" s="25" t="s"/>
-      <c r="E13" s="25" t="s"/>
-      <c r="F13" s="25" t="s"/>
-      <c r="G13" s="25" t="s"/>
-      <c r="H13" s="17" t="s"/>
-      <c r="I13" s="10" t="s"/>
-      <c r="J13" s="10" t="s"/>
-      <c r="K13" s="25" t="s"/>
-      <c r="L13" s="24" t="s"/>
-      <c r="M13" s="24" t="s"/>
+      <c r="B13" s="25">
+        <v>10</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="D13" s="25">
+        <v>2</v>
+      </c>
+      <c r="E13" s="25">
+        <v>32</v>
+      </c>
+      <c r="F13" s="25">
+        <v>24</v>
+      </c>
+      <c r="G13" s="25">
+        <v>14</v>
+      </c>
+      <c r="H13" s="17">
+        <v>0</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="K13" s="25">
+        <v>1000</v>
+      </c>
+      <c r="L13" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="M13" s="24">
+        <v>3</v>
+      </c>
     </row>
     <row r="14" spans="1:13" ht="39.95" customHeight="1">
       <c r="A14" s="17" t="s"/>
-      <c r="B14" s="25" t="s"/>
-      <c r="C14" s="10" t="s"/>
-      <c r="D14" s="25" t="s"/>
-      <c r="E14" s="25" t="s"/>
-      <c r="F14" s="25" t="s"/>
-      <c r="G14" s="25" t="s"/>
-      <c r="H14" s="17" t="s"/>
-      <c r="I14" s="10" t="s"/>
-      <c r="J14" s="10" t="s"/>
-      <c r="K14" s="25" t="s"/>
-      <c r="L14" s="24" t="s"/>
-      <c r="M14" s="24" t="s"/>
+      <c r="B14" s="25">
+        <v>11</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="D14" s="25">
+        <v>3</v>
+      </c>
+      <c r="E14" s="25">
+        <v>48</v>
+      </c>
+      <c r="F14" s="25">
+        <v>38</v>
+      </c>
+      <c r="G14" s="25">
+        <v>10</v>
+      </c>
+      <c r="H14" s="17">
+        <v>0</v>
+      </c>
+      <c r="I14" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="J14" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="K14" s="25">
+        <v>800</v>
+      </c>
+      <c r="L14" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="M14" s="24">
+        <v>3</v>
+      </c>
     </row>
     <row r="15" spans="1:13" ht="39.95" customHeight="1">
       <c r="A15" s="17" t="s"/>
-      <c r="B15" s="25" t="s"/>
-      <c r="C15" s="10" t="s"/>
-      <c r="D15" s="25" t="s"/>
-      <c r="E15" s="25" t="s"/>
-      <c r="F15" s="25" t="s"/>
-      <c r="G15" s="25" t="s"/>
-      <c r="H15" s="17" t="s"/>
-      <c r="I15" s="10" t="s"/>
-      <c r="J15" s="10" t="s"/>
-      <c r="K15" s="25" t="s"/>
-      <c r="L15" s="24" t="s"/>
-      <c r="M15" s="24" t="s"/>
+      <c r="B15" s="25">
+        <v>12</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="D15" s="25">
+        <v>4</v>
+      </c>
+      <c r="E15" s="25">
+        <v>72</v>
+      </c>
+      <c r="F15" s="25">
+        <v>62</v>
+      </c>
+      <c r="G15" s="25">
+        <v>8</v>
+      </c>
+      <c r="H15" s="17">
+        <v>0</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="J15" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="K15" s="25">
+        <v>600</v>
+      </c>
+      <c r="L15" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="M15" s="24">
+        <v>3</v>
+      </c>
     </row>
     <row r="16" spans="1:13" ht="39.95" customHeight="1">
       <c r="A16" s="17" t="s"/>
-      <c r="B16" s="25" t="s"/>
-      <c r="C16" s="10" t="s"/>
-      <c r="D16" s="25" t="s"/>
-      <c r="E16" s="25" t="s"/>
-      <c r="F16" s="25" t="s"/>
-      <c r="G16" s="25" t="s"/>
-      <c r="H16" s="17" t="s"/>
-      <c r="I16" s="10" t="s"/>
-      <c r="J16" s="10" t="s"/>
-      <c r="K16" s="25" t="s"/>
-      <c r="L16" s="24" t="s"/>
-      <c r="M16" s="24" t="s"/>
+      <c r="B16" s="25">
+        <v>13</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="D16" s="25">
+        <v>3</v>
+      </c>
+      <c r="E16" s="25">
+        <v>48</v>
+      </c>
+      <c r="F16" s="25">
+        <v>38</v>
+      </c>
+      <c r="G16" s="25">
+        <v>10</v>
+      </c>
+      <c r="H16" s="17">
+        <v>0</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="J16" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="K16" s="25">
+        <v>800</v>
+      </c>
+      <c r="L16" s="24" t="s">
+        <v>133</v>
+      </c>
+      <c r="M16" s="24">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" spans="1:13" ht="39.95" customHeight="1">
       <c r="A17" s="17" t="s"/>
-      <c r="B17" s="25" t="s"/>
-      <c r="C17" s="10" t="s"/>
-      <c r="D17" s="25" t="s"/>
-      <c r="E17" s="25" t="s"/>
-      <c r="F17" s="25" t="s"/>
-      <c r="G17" s="25" t="s"/>
-      <c r="H17" s="17" t="s"/>
-      <c r="I17" s="10" t="s"/>
-      <c r="J17" s="10" t="s"/>
-      <c r="K17" s="25" t="s"/>
-      <c r="L17" s="24" t="s"/>
-      <c r="M17" s="24" t="s"/>
+      <c r="B17" s="25">
+        <v>14</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="D17" s="25">
+        <v>4</v>
+      </c>
+      <c r="E17" s="25">
+        <v>72</v>
+      </c>
+      <c r="F17" s="25">
+        <v>62</v>
+      </c>
+      <c r="G17" s="25">
+        <v>8</v>
+      </c>
+      <c r="H17" s="17">
+        <v>0</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="J17" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="K17" s="25">
+        <v>600</v>
+      </c>
+      <c r="L17" s="24" t="s">
+        <v>136</v>
+      </c>
+      <c r="M17" s="24">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" spans="1:13" ht="39.95" customHeight="1">
       <c r="A18" s="17" t="s"/>
-      <c r="B18" s="25" t="s"/>
-      <c r="C18" s="10" t="s"/>
-      <c r="D18" s="25" t="s"/>
-      <c r="E18" s="25" t="s"/>
-      <c r="F18" s="25" t="s"/>
-      <c r="G18" s="25" t="s"/>
-      <c r="H18" s="17" t="s"/>
-      <c r="I18" s="10" t="s"/>
-      <c r="J18" s="10" t="s"/>
-      <c r="K18" s="25" t="s"/>
-      <c r="L18" s="24" t="s"/>
-      <c r="M18" s="24" t="s"/>
+      <c r="B18" s="25">
+        <v>15</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D18" s="25">
+        <v>5</v>
+      </c>
+      <c r="E18" s="25">
+        <v>80</v>
+      </c>
+      <c r="F18" s="25">
+        <v>70</v>
+      </c>
+      <c r="G18" s="25">
+        <v>30</v>
+      </c>
+      <c r="H18" s="17">
+        <v>0</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="J18" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="K18" s="25">
+        <v>800</v>
+      </c>
+      <c r="L18" s="24" t="s">
+        <v>139</v>
+      </c>
+      <c r="M18" s="24">
+        <v>1</v>
+      </c>
     </row>
     <row r="19" spans="1:11" ht="39.95" customHeight="1">
       <c r="A19" s="14" t="s"/>

</xml_diff>